<commit_message>
feat: Update RF Switch Tool with new report generation and testing features
- Added new HTML report generation for RF Switch Tool with detailed summaries and visualizations.
- Introduced a new PNG chart for test statistics.
- Updated configuration to reflect new button IDs and window title.
- Enhanced Excel logging functionality to support dynamic sheet names based on test type.
- Improved data visualization in reports with better styling and layout.
- Fixed issues with button interaction tests and logging to ensure accurate data capture.
- Added new HTML report for v8000 with comprehensive test results.
</commit_message>
<xml_diff>
--- a/RF_All_Tests_Results_20260624.xlsx
+++ b/RF_All_Tests_Results_20260624.xlsx
@@ -7,7 +7,9 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="測試結果" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="常規規律測試" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="特殊規律測試" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="單鈕互動測試" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -413,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G41"/>
+  <dimension ref="A1:G17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -461,7 +463,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>第 1 步 (鈕 1)</t>
+          <t>第 1 步</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -470,17 +472,17 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>0.07000000000000001</v>
+        <v>0.2</v>
       </c>
       <c r="E2" t="n">
-        <v>186.35</v>
+        <v>160.93</v>
       </c>
       <c r="F2" t="n">
-        <v>186.35</v>
+        <v>160.93</v>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>2026-06-24 11:34:53</t>
+          <t>2026-06-24 11:56:38</t>
         </is>
       </c>
     </row>
@@ -492,7 +494,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>第 2 步 (鈕 2)</t>
+          <t>第 2 步</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -501,17 +503,17 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>109.72</v>
+        <v>111.99</v>
       </c>
       <c r="E3" t="n">
-        <v>109.72</v>
+        <v>111.99</v>
       </c>
       <c r="F3" t="n">
-        <v>109.72</v>
+        <v>111.99</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>2026-06-24 11:34:55</t>
+          <t>2026-06-24 11:56:40</t>
         </is>
       </c>
     </row>
@@ -523,26 +525,26 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>第 3 步 (鈕 1)</t>
+          <t>第 3 步</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>CheckBox28_1</t>
+          <t>CheckBox28_3</t>
         </is>
       </c>
       <c r="D4" t="n">
-        <v>109.73</v>
+        <v>53.51</v>
       </c>
       <c r="E4" t="n">
-        <v>109.73</v>
+        <v>102.4</v>
       </c>
       <c r="F4" t="n">
-        <v>109.73</v>
+        <v>102.4</v>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>2026-06-24 11:34:56</t>
+          <t>2026-06-24 11:56:41</t>
         </is>
       </c>
     </row>
@@ -554,26 +556,26 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>第 4 步 (鈕 3)</t>
+          <t>第 4 步</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>CheckBox28_3</t>
+          <t>CheckBox28_4</t>
         </is>
       </c>
       <c r="D5" t="n">
-        <v>56.8</v>
+        <v>109.74</v>
       </c>
       <c r="E5" t="n">
-        <v>56.8</v>
+        <v>109.74</v>
       </c>
       <c r="F5" t="n">
-        <v>56.8</v>
+        <v>109.74</v>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>2026-06-24 11:34:57</t>
+          <t>2026-06-24 11:56:42</t>
         </is>
       </c>
     </row>
@@ -585,26 +587,26 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>第 5 步 (鈕 4)</t>
+          <t>第 5 步</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>CheckBox28_4</t>
+          <t>CheckBox28_5</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>110.89</v>
+        <v>52.83</v>
       </c>
       <c r="E6" t="n">
-        <v>160.4</v>
+        <v>110.22</v>
       </c>
       <c r="F6" t="n">
-        <v>160.4</v>
+        <v>110.22</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>2026-06-24 11:34:59</t>
+          <t>2026-06-24 11:56:43</t>
         </is>
       </c>
     </row>
@@ -616,26 +618,26 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>第 6 步 (鈕 3)</t>
+          <t>第 6 步</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>CheckBox28_3</t>
+          <t>CheckBox28_6</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>60.51</v>
+        <v>111.83</v>
       </c>
       <c r="E7" t="n">
-        <v>107.97</v>
+        <v>111.83</v>
       </c>
       <c r="F7" t="n">
-        <v>107.97</v>
+        <v>111.83</v>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>2026-06-24 11:35:00</t>
+          <t>2026-06-24 11:56:45</t>
         </is>
       </c>
     </row>
@@ -647,26 +649,26 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>第 7 步 (鈕 5)</t>
+          <t>第 7 步</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>CheckBox28_5</t>
+          <t>CheckBox28_7</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>55.14</v>
+        <v>110.45</v>
       </c>
       <c r="E8" t="n">
-        <v>103.8</v>
+        <v>110.45</v>
       </c>
       <c r="F8" t="n">
-        <v>103.8</v>
+        <v>110.45</v>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>2026-06-24 11:35:01</t>
+          <t>2026-06-24 11:56:46</t>
         </is>
       </c>
     </row>
@@ -678,150 +680,150 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>第 8 步 (鈕 6)</t>
+          <t>第 8 步</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>CheckBox28_6</t>
+          <t>CheckBox28_8</t>
         </is>
       </c>
       <c r="D9" t="n">
-        <v>113.95</v>
+        <v>54.23</v>
       </c>
       <c r="E9" t="n">
-        <v>113.95</v>
+        <v>54.23</v>
       </c>
       <c r="F9" t="n">
-        <v>113.95</v>
+        <v>54.23</v>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>2026-06-24 11:35:03</t>
+          <t>2026-06-24 11:56:47</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>第 1 輪</t>
+          <t>第 2 輪</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>第 9 步 (鈕 5)</t>
+          <t>第 1 步</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>CheckBox28_5</t>
+          <t>CheckBox28_1</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>109.97</v>
+        <v>110.64</v>
       </c>
       <c r="E10" t="n">
-        <v>109.97</v>
+        <v>110.64</v>
       </c>
       <c r="F10" t="n">
-        <v>109.97</v>
+        <v>110.64</v>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>2026-06-24 11:35:04</t>
+          <t>2026-06-24 11:56:49</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>第 1 輪</t>
+          <t>第 2 輪</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>第 10 步 (鈕 7)</t>
+          <t>第 2 步</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>CheckBox28_7</t>
+          <t>CheckBox28_2</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>114.96</v>
+        <v>57.75</v>
       </c>
       <c r="E11" t="n">
-        <v>114.96</v>
+        <v>113.77</v>
       </c>
       <c r="F11" t="n">
-        <v>114.96</v>
+        <v>113.77</v>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>2026-06-24 11:35:05</t>
+          <t>2026-06-24 11:56:50</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>第 1 輪</t>
+          <t>第 2 輪</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>第 11 步 (鈕 8)</t>
+          <t>第 3 步</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>CheckBox28_8</t>
+          <t>CheckBox28_3</t>
         </is>
       </c>
       <c r="D12" t="n">
-        <v>0.06</v>
+        <v>108.9</v>
       </c>
       <c r="E12" t="n">
-        <v>47.64</v>
+        <v>108.9</v>
       </c>
       <c r="F12" t="n">
-        <v>47.64</v>
+        <v>108.9</v>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>2026-06-24 11:35:07</t>
+          <t>2026-06-24 11:56:51</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>第 1 輪</t>
+          <t>第 2 輪</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>第 12 步 (鈕 7)</t>
+          <t>第 4 步</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>CheckBox28_7</t>
+          <t>CheckBox28_4</t>
         </is>
       </c>
       <c r="D13" t="n">
-        <v>0.05</v>
+        <v>55.88</v>
       </c>
       <c r="E13" t="n">
-        <v>133.2</v>
+        <v>103.76</v>
       </c>
       <c r="F13" t="n">
-        <v>133.2</v>
+        <v>103.76</v>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>2026-06-24 11:35:08</t>
+          <t>2026-06-24 11:56:53</t>
         </is>
       </c>
     </row>
@@ -833,26 +835,26 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>第 1 步 (鈕 1)</t>
+          <t>第 5 步</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>CheckBox28_1</t>
+          <t>CheckBox28_5</t>
         </is>
       </c>
       <c r="D14" t="n">
-        <v>56.84</v>
+        <v>111.98</v>
       </c>
       <c r="E14" t="n">
-        <v>105.73</v>
+        <v>111.98</v>
       </c>
       <c r="F14" t="n">
-        <v>105.73</v>
+        <v>111.98</v>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>2026-06-24 11:35:09</t>
+          <t>2026-06-24 11:56:54</t>
         </is>
       </c>
     </row>
@@ -864,26 +866,26 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>第 2 步 (鈕 2)</t>
+          <t>第 6 步</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>CheckBox28_2</t>
+          <t>CheckBox28_6</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>54.53</v>
+        <v>111.02</v>
       </c>
       <c r="E15" t="n">
-        <v>102.65</v>
+        <v>111.02</v>
       </c>
       <c r="F15" t="n">
-        <v>102.65</v>
+        <v>111.02</v>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>2026-06-24 11:35:10</t>
+          <t>2026-06-24 11:56:55</t>
         </is>
       </c>
     </row>
@@ -895,26 +897,26 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>第 3 步 (鈕 1)</t>
+          <t>第 7 步</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>CheckBox28_1</t>
+          <t>CheckBox28_7</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>110.15</v>
+        <v>110.53</v>
       </c>
       <c r="E16" t="n">
-        <v>110.15</v>
+        <v>110.53</v>
       </c>
       <c r="F16" t="n">
-        <v>110.15</v>
+        <v>110.53</v>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>2026-06-24 11:35:12</t>
+          <t>2026-06-24 11:56:56</t>
         </is>
       </c>
     </row>
@@ -926,26 +928,573 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
+          <t>第 8 步</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>CheckBox28_8</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>55.16</v>
+      </c>
+      <c r="E17" t="n">
+        <v>103.72</v>
+      </c>
+      <c r="F17" t="n">
+        <v>103.72</v>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>2026-06-24 11:56:58</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G25"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>輪次</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>邏輯順序</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>按鈕實體ID</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>前鈕恢復時間(ms)</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>新鈕變色時間(ms)</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>總耗時(ms)</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>測試時間</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>第 1 輪</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>第 1 步 (鈕 1)</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>CheckBox28_1</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="E2" t="n">
+        <v>212.51</v>
+      </c>
+      <c r="F2" t="n">
+        <v>212.51</v>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>2026-06-24 11:57:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>第 1 輪</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>第 2 步 (鈕 2)</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>CheckBox28_2</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>110.66</v>
+      </c>
+      <c r="E3" t="n">
+        <v>110.66</v>
+      </c>
+      <c r="F3" t="n">
+        <v>110.66</v>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>2026-06-24 11:57:02</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>第 1 輪</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>第 3 步 (鈕 1)</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>CheckBox28_1</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>109.29</v>
+      </c>
+      <c r="E4" t="n">
+        <v>109.29</v>
+      </c>
+      <c r="F4" t="n">
+        <v>109.29</v>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>2026-06-24 11:57:03</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>第 1 輪</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
           <t>第 4 步 (鈕 3)</t>
         </is>
       </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>CheckBox28_3</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>53.95</v>
+      </c>
+      <c r="E5" t="n">
+        <v>102.41</v>
+      </c>
+      <c r="F5" t="n">
+        <v>102.41</v>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>2026-06-24 11:57:04</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>第 1 輪</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>第 5 步 (鈕 4)</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>CheckBox28_4</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>55.3</v>
+      </c>
+      <c r="E6" t="n">
+        <v>102.62</v>
+      </c>
+      <c r="F6" t="n">
+        <v>102.62</v>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>2026-06-24 11:57:06</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>第 1 輪</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>第 6 步 (鈕 3)</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>CheckBox28_3</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>57.84</v>
+      </c>
+      <c r="E7" t="n">
+        <v>114.5</v>
+      </c>
+      <c r="F7" t="n">
+        <v>114.5</v>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>2026-06-24 11:57:07</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>第 1 輪</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>第 7 步 (鈕 5)</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>CheckBox28_5</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>107.75</v>
+      </c>
+      <c r="E8" t="n">
+        <v>107.75</v>
+      </c>
+      <c r="F8" t="n">
+        <v>107.75</v>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>2026-06-24 11:57:08</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>第 1 輪</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>第 8 步 (鈕 6)</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>CheckBox28_6</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>57.15</v>
+      </c>
+      <c r="E9" t="n">
+        <v>105.96</v>
+      </c>
+      <c r="F9" t="n">
+        <v>105.96</v>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>2026-06-24 11:57:09</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>第 1 輪</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>第 9 步 (鈕 5)</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>CheckBox28_5</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>109.35</v>
+      </c>
+      <c r="E10" t="n">
+        <v>109.35</v>
+      </c>
+      <c r="F10" t="n">
+        <v>109.35</v>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>2026-06-24 11:57:11</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>第 1 輪</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>第 10 步 (鈕 7)</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>CheckBox28_7</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>112.18</v>
+      </c>
+      <c r="E11" t="n">
+        <v>112.18</v>
+      </c>
+      <c r="F11" t="n">
+        <v>112.18</v>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>2026-06-24 11:57:12</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>第 1 輪</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>第 11 步 (鈕 8)</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>CheckBox28_8</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>108.52</v>
+      </c>
+      <c r="E12" t="n">
+        <v>108.52</v>
+      </c>
+      <c r="F12" t="n">
+        <v>108.52</v>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>2026-06-24 11:57:13</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>第 1 輪</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>第 12 步 (鈕 7)</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>CheckBox28_7</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>54.66</v>
+      </c>
+      <c r="E13" t="n">
+        <v>103.32</v>
+      </c>
+      <c r="F13" t="n">
+        <v>103.32</v>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>2026-06-24 11:57:15</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>第 2 輪</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>第 1 步 (鈕 1)</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>CheckBox28_1</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>58.82</v>
+      </c>
+      <c r="E14" t="n">
+        <v>106.77</v>
+      </c>
+      <c r="F14" t="n">
+        <v>106.77</v>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>2026-06-24 11:57:16</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>第 2 輪</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>第 2 步 (鈕 2)</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>CheckBox28_2</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>52.84</v>
+      </c>
+      <c r="E15" t="n">
+        <v>102.35</v>
+      </c>
+      <c r="F15" t="n">
+        <v>102.35</v>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>2026-06-24 11:57:17</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>第 2 輪</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>第 3 步 (鈕 1)</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>CheckBox28_1</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>54.68</v>
+      </c>
+      <c r="E16" t="n">
+        <v>103.02</v>
+      </c>
+      <c r="F16" t="n">
+        <v>103.02</v>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>2026-06-24 11:57:19</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>第 2 輪</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>第 4 步 (鈕 3)</t>
+        </is>
+      </c>
       <c r="C17" t="inlineStr">
         <is>
           <t>CheckBox28_3</t>
         </is>
       </c>
       <c r="D17" t="n">
-        <v>55.25</v>
+        <v>54.93</v>
       </c>
       <c r="E17" t="n">
-        <v>109.62</v>
+        <v>111.7</v>
       </c>
       <c r="F17" t="n">
-        <v>109.62</v>
+        <v>111.7</v>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>2026-06-24 11:35:13</t>
+          <t>2026-06-24 11:57:20</t>
         </is>
       </c>
     </row>
@@ -966,17 +1515,17 @@
         </is>
       </c>
       <c r="D18" t="n">
-        <v>110.86</v>
+        <v>52.53</v>
       </c>
       <c r="E18" t="n">
-        <v>110.86</v>
+        <v>101.09</v>
       </c>
       <c r="F18" t="n">
-        <v>110.86</v>
+        <v>101.09</v>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>2026-06-24 11:35:14</t>
+          <t>2026-06-24 11:57:21</t>
         </is>
       </c>
     </row>
@@ -997,17 +1546,17 @@
         </is>
       </c>
       <c r="D19" t="n">
-        <v>57.12</v>
+        <v>53.68</v>
       </c>
       <c r="E19" t="n">
-        <v>104.47</v>
+        <v>108.66</v>
       </c>
       <c r="F19" t="n">
-        <v>104.47</v>
+        <v>108.66</v>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>2026-06-24 11:35:16</t>
+          <t>2026-06-24 11:57:22</t>
         </is>
       </c>
     </row>
@@ -1028,17 +1577,17 @@
         </is>
       </c>
       <c r="D20" t="n">
-        <v>108.77</v>
+        <v>112.53</v>
       </c>
       <c r="E20" t="n">
-        <v>108.77</v>
+        <v>112.53</v>
       </c>
       <c r="F20" t="n">
-        <v>108.77</v>
+        <v>112.53</v>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>2026-06-24 11:35:17</t>
+          <t>2026-06-24 11:57:24</t>
         </is>
       </c>
     </row>
@@ -1059,17 +1608,17 @@
         </is>
       </c>
       <c r="D21" t="n">
-        <v>108.93</v>
+        <v>59.28</v>
       </c>
       <c r="E21" t="n">
-        <v>108.93</v>
+        <v>107.5</v>
       </c>
       <c r="F21" t="n">
-        <v>108.93</v>
+        <v>107.5</v>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>2026-06-24 11:35:18</t>
+          <t>2026-06-24 11:57:25</t>
         </is>
       </c>
     </row>
@@ -1090,17 +1639,17 @@
         </is>
       </c>
       <c r="D22" t="n">
-        <v>111.24</v>
+        <v>108.04</v>
       </c>
       <c r="E22" t="n">
-        <v>111.24</v>
+        <v>108.04</v>
       </c>
       <c r="F22" t="n">
-        <v>111.24</v>
+        <v>108.04</v>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>2026-06-24 11:35:20</t>
+          <t>2026-06-24 11:57:26</t>
         </is>
       </c>
     </row>
@@ -1121,17 +1670,17 @@
         </is>
       </c>
       <c r="D23" t="n">
-        <v>57.39</v>
+        <v>55.58</v>
       </c>
       <c r="E23" t="n">
-        <v>106.89</v>
+        <v>104.06</v>
       </c>
       <c r="F23" t="n">
-        <v>106.89</v>
+        <v>104.06</v>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>2026-06-24 11:35:21</t>
+          <t>2026-06-24 11:57:28</t>
         </is>
       </c>
     </row>
@@ -1152,17 +1701,17 @@
         </is>
       </c>
       <c r="D24" t="n">
-        <v>54.14</v>
+        <v>53.92</v>
       </c>
       <c r="E24" t="n">
-        <v>102.4</v>
+        <v>103.28</v>
       </c>
       <c r="F24" t="n">
-        <v>102.4</v>
+        <v>103.28</v>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>2026-06-24 11:35:22</t>
+          <t>2026-06-24 11:57:29</t>
         </is>
       </c>
     </row>
@@ -1183,513 +1732,564 @@
         </is>
       </c>
       <c r="D25" t="n">
-        <v>109.21</v>
+        <v>55.41</v>
       </c>
       <c r="E25" t="n">
-        <v>156.14</v>
+        <v>104.06</v>
       </c>
       <c r="F25" t="n">
-        <v>156.14</v>
+        <v>104.06</v>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>2026-06-24 11:35:23</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t>第 1 輪</t>
-        </is>
-      </c>
-      <c r="B26" t="inlineStr">
+          <t>2026-06-24 11:57:30</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G17"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>輪次</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>按鈕實體ID</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>識別代碼</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>變藍耗時(ms)</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>變灰耗時(ms)</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>總耗時(ms)</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>測試時間</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>第 1 輪</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
         <is>
           <t>按鈕 1</t>
         </is>
       </c>
-      <c r="C26" t="inlineStr">
+      <c r="C2" t="inlineStr">
         <is>
           <t>CheckBox28_1</t>
         </is>
       </c>
-      <c r="D26" t="n">
+      <c r="D2" t="n">
         <v>0</v>
       </c>
-      <c r="E26" t="n">
+      <c r="E2" t="n">
         <v>0</v>
       </c>
-      <c r="F26" t="n">
+      <c r="F2" t="n">
         <v>0.01</v>
       </c>
-      <c r="G26" t="inlineStr">
-        <is>
-          <t>2026-06-24 11:35:26</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t>第 1 輪</t>
-        </is>
-      </c>
-      <c r="B27" t="inlineStr">
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>2026-06-24 11:57:33</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>第 1 輪</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
         <is>
           <t>按鈕 2</t>
         </is>
       </c>
-      <c r="C27" t="inlineStr">
+      <c r="C3" t="inlineStr">
         <is>
           <t>CheckBox28_2</t>
         </is>
       </c>
-      <c r="D27" t="n">
-        <v>85.69</v>
-      </c>
-      <c r="E27" t="n">
+      <c r="D3" t="n">
+        <v>57.17</v>
+      </c>
+      <c r="E3" t="n">
         <v>0</v>
       </c>
-      <c r="F27" t="n">
-        <v>85.69</v>
-      </c>
-      <c r="G27" t="inlineStr">
-        <is>
-          <t>2026-06-24 11:35:29</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t>第 1 輪</t>
-        </is>
-      </c>
-      <c r="B28" t="inlineStr">
+      <c r="F3" t="n">
+        <v>57.18</v>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>2026-06-24 11:57:35</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>第 1 輪</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
         <is>
           <t>按鈕 3</t>
         </is>
       </c>
-      <c r="C28" t="inlineStr">
+      <c r="C4" t="inlineStr">
         <is>
           <t>CheckBox28_3</t>
         </is>
       </c>
-      <c r="D28" t="n">
-        <v>56.2</v>
-      </c>
-      <c r="E28" t="n">
+      <c r="D4" t="n">
+        <v>52.71</v>
+      </c>
+      <c r="E4" t="n">
         <v>0</v>
       </c>
-      <c r="F28" t="n">
-        <v>56.2</v>
-      </c>
-      <c r="G28" t="inlineStr">
-        <is>
-          <t>2026-06-24 11:35:31</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>第 1 輪</t>
-        </is>
-      </c>
-      <c r="B29" t="inlineStr">
+      <c r="F4" t="n">
+        <v>52.72</v>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>2026-06-24 11:57:38</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>第 1 輪</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
         <is>
           <t>按鈕 4</t>
         </is>
       </c>
-      <c r="C29" t="inlineStr">
+      <c r="C5" t="inlineStr">
         <is>
           <t>CheckBox28_4</t>
         </is>
       </c>
-      <c r="D29" t="n">
-        <v>83.33</v>
-      </c>
-      <c r="E29" t="n">
+      <c r="D5" t="n">
+        <v>24.21</v>
+      </c>
+      <c r="E5" t="n">
         <v>0</v>
       </c>
-      <c r="F29" t="n">
-        <v>83.33</v>
-      </c>
-      <c r="G29" t="inlineStr">
-        <is>
-          <t>2026-06-24 11:35:34</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" t="inlineStr">
-        <is>
-          <t>第 1 輪</t>
-        </is>
-      </c>
-      <c r="B30" t="inlineStr">
+      <c r="F5" t="n">
+        <v>24.21</v>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>2026-06-24 11:57:41</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>第 1 輪</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
         <is>
           <t>按鈕 5</t>
         </is>
       </c>
-      <c r="C30" t="inlineStr">
+      <c r="C6" t="inlineStr">
         <is>
           <t>CheckBox28_5</t>
         </is>
       </c>
-      <c r="D30" t="n">
-        <v>81.75</v>
-      </c>
-      <c r="E30" t="n">
-        <v>0.01</v>
-      </c>
-      <c r="F30" t="n">
-        <v>81.76000000000001</v>
-      </c>
-      <c r="G30" t="inlineStr">
-        <is>
-          <t>2026-06-24 11:35:37</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" t="inlineStr">
-        <is>
-          <t>第 1 輪</t>
-        </is>
-      </c>
-      <c r="B31" t="inlineStr">
+      <c r="D6" t="n">
+        <v>30.08</v>
+      </c>
+      <c r="E6" t="n">
+        <v>0</v>
+      </c>
+      <c r="F6" t="n">
+        <v>30.08</v>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>2026-06-24 11:57:43</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>第 1 輪</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
         <is>
           <t>按鈕 6</t>
         </is>
       </c>
-      <c r="C31" t="inlineStr">
+      <c r="C7" t="inlineStr">
         <is>
           <t>CheckBox28_6</t>
         </is>
       </c>
-      <c r="D31" t="n">
-        <v>26.67</v>
-      </c>
-      <c r="E31" t="n">
+      <c r="D7" t="n">
+        <v>26.22</v>
+      </c>
+      <c r="E7" t="n">
         <v>0</v>
       </c>
-      <c r="F31" t="n">
-        <v>26.67</v>
-      </c>
-      <c r="G31" t="inlineStr">
-        <is>
-          <t>2026-06-24 11:35:39</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" t="inlineStr">
-        <is>
-          <t>第 1 輪</t>
-        </is>
-      </c>
-      <c r="B32" t="inlineStr">
+      <c r="F7" t="n">
+        <v>26.23</v>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>2026-06-24 11:57:46</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>第 1 輪</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
         <is>
           <t>按鈕 7</t>
         </is>
       </c>
-      <c r="C32" t="inlineStr">
+      <c r="C8" t="inlineStr">
         <is>
           <t>CheckBox28_7</t>
         </is>
       </c>
-      <c r="D32" t="n">
-        <v>85.18000000000001</v>
-      </c>
-      <c r="E32" t="n">
+      <c r="D8" t="n">
+        <v>56.01</v>
+      </c>
+      <c r="E8" t="n">
         <v>0</v>
       </c>
-      <c r="F32" t="n">
-        <v>85.18000000000001</v>
-      </c>
-      <c r="G32" t="inlineStr">
-        <is>
-          <t>2026-06-24 11:35:42</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" t="inlineStr">
-        <is>
-          <t>第 1 輪</t>
-        </is>
-      </c>
-      <c r="B33" t="inlineStr">
+      <c r="F8" t="n">
+        <v>56.01</v>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>2026-06-24 11:57:48</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>第 1 輪</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
         <is>
           <t>按鈕 8</t>
         </is>
       </c>
-      <c r="C33" t="inlineStr">
+      <c r="C9" t="inlineStr">
         <is>
           <t>CheckBox28_8</t>
         </is>
       </c>
-      <c r="D33" t="n">
-        <v>110.54</v>
-      </c>
-      <c r="E33" t="n">
+      <c r="D9" t="n">
+        <v>55.16</v>
+      </c>
+      <c r="E9" t="n">
         <v>0</v>
       </c>
-      <c r="F33" t="n">
-        <v>110.54</v>
-      </c>
-      <c r="G33" t="inlineStr">
-        <is>
-          <t>2026-06-24 11:35:44</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" t="inlineStr">
-        <is>
-          <t>第 2 輪</t>
-        </is>
-      </c>
-      <c r="B34" t="inlineStr">
+      <c r="F9" t="n">
+        <v>55.16</v>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>2026-06-24 11:57:51</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>第 2 輪</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
         <is>
           <t>按鈕 1</t>
         </is>
       </c>
-      <c r="C34" t="inlineStr">
+      <c r="C10" t="inlineStr">
         <is>
           <t>CheckBox28_1</t>
         </is>
       </c>
-      <c r="D34" t="n">
-        <v>85.29000000000001</v>
-      </c>
-      <c r="E34" t="n">
+      <c r="D10" t="n">
+        <v>81.65000000000001</v>
+      </c>
+      <c r="E10" t="n">
         <v>0</v>
       </c>
-      <c r="F34" t="n">
-        <v>85.29000000000001</v>
-      </c>
-      <c r="G34" t="inlineStr">
-        <is>
-          <t>2026-06-24 11:35:47</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" t="inlineStr">
-        <is>
-          <t>第 2 輪</t>
-        </is>
-      </c>
-      <c r="B35" t="inlineStr">
+      <c r="F10" t="n">
+        <v>81.65000000000001</v>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>2026-06-24 11:57:54</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>第 2 輪</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
         <is>
           <t>按鈕 2</t>
         </is>
       </c>
-      <c r="C35" t="inlineStr">
+      <c r="C11" t="inlineStr">
         <is>
           <t>CheckBox28_2</t>
         </is>
       </c>
-      <c r="D35" t="n">
-        <v>108.83</v>
-      </c>
-      <c r="E35" t="n">
+      <c r="D11" t="n">
+        <v>23.64</v>
+      </c>
+      <c r="E11" t="n">
         <v>0</v>
       </c>
-      <c r="F35" t="n">
-        <v>108.84</v>
-      </c>
-      <c r="G35" t="inlineStr">
-        <is>
-          <t>2026-06-24 11:35:50</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" t="inlineStr">
-        <is>
-          <t>第 2 輪</t>
-        </is>
-      </c>
-      <c r="B36" t="inlineStr">
+      <c r="F11" t="n">
+        <v>23.65</v>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>2026-06-24 11:57:56</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>第 2 輪</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
         <is>
           <t>按鈕 3</t>
         </is>
       </c>
-      <c r="C36" t="inlineStr">
+      <c r="C12" t="inlineStr">
         <is>
           <t>CheckBox28_3</t>
         </is>
       </c>
-      <c r="D36" t="n">
-        <v>81.42</v>
-      </c>
-      <c r="E36" t="n">
+      <c r="D12" t="n">
+        <v>58.75</v>
+      </c>
+      <c r="E12" t="n">
         <v>0</v>
       </c>
-      <c r="F36" t="n">
-        <v>81.42</v>
-      </c>
-      <c r="G36" t="inlineStr">
-        <is>
-          <t>2026-06-24 11:35:52</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" t="inlineStr">
-        <is>
-          <t>第 2 輪</t>
-        </is>
-      </c>
-      <c r="B37" t="inlineStr">
+      <c r="F12" t="n">
+        <v>58.75</v>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>2026-06-24 11:57:59</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>第 2 輪</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
         <is>
           <t>按鈕 4</t>
         </is>
       </c>
-      <c r="C37" t="inlineStr">
+      <c r="C13" t="inlineStr">
         <is>
           <t>CheckBox28_4</t>
         </is>
       </c>
-      <c r="D37" t="n">
-        <v>81.91</v>
-      </c>
-      <c r="E37" t="n">
+      <c r="D13" t="n">
+        <v>56.82</v>
+      </c>
+      <c r="E13" t="n">
+        <v>111.74</v>
+      </c>
+      <c r="F13" t="n">
+        <v>168.56</v>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>2026-06-24 11:58:02</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>第 2 輪</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>按鈕 5</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>CheckBox28_5</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>137.75</v>
+      </c>
+      <c r="E14" t="n">
         <v>0</v>
       </c>
-      <c r="F37" t="n">
-        <v>81.91</v>
-      </c>
-      <c r="G37" t="inlineStr">
-        <is>
-          <t>2026-06-24 11:35:55</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" t="inlineStr">
-        <is>
-          <t>第 2 輪</t>
-        </is>
-      </c>
-      <c r="B38" t="inlineStr">
-        <is>
-          <t>按鈕 5</t>
-        </is>
-      </c>
-      <c r="C38" t="inlineStr">
-        <is>
-          <t>CheckBox28_5</t>
-        </is>
-      </c>
-      <c r="D38" t="n">
-        <v>56.98</v>
-      </c>
-      <c r="E38" t="n">
+      <c r="F14" t="n">
+        <v>137.75</v>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>2026-06-24 11:58:04</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>第 2 輪</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>按鈕 6</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>CheckBox28_6</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
         <v>0</v>
       </c>
-      <c r="F38" t="n">
-        <v>56.98</v>
-      </c>
-      <c r="G38" t="inlineStr">
-        <is>
-          <t>2026-06-24 11:35:57</t>
-        </is>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" t="inlineStr">
-        <is>
-          <t>第 2 輪</t>
-        </is>
-      </c>
-      <c r="B39" t="inlineStr">
-        <is>
-          <t>按鈕 6</t>
-        </is>
-      </c>
-      <c r="C39" t="inlineStr">
-        <is>
-          <t>CheckBox28_6</t>
-        </is>
-      </c>
-      <c r="D39" t="n">
-        <v>83.68000000000001</v>
-      </c>
-      <c r="E39" t="n">
+      <c r="E15" t="n">
         <v>0</v>
       </c>
-      <c r="F39" t="n">
-        <v>83.68000000000001</v>
-      </c>
-      <c r="G39" t="inlineStr">
-        <is>
-          <t>2026-06-24 11:36:00</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" t="inlineStr">
-        <is>
-          <t>第 2 輪</t>
-        </is>
-      </c>
-      <c r="B40" t="inlineStr">
+      <c r="F15" t="n">
+        <v>0</v>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>2026-06-24 11:58:07</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>第 2 輪</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
         <is>
           <t>按鈕 7</t>
         </is>
       </c>
-      <c r="C40" t="inlineStr">
+      <c r="C16" t="inlineStr">
         <is>
           <t>CheckBox28_7</t>
         </is>
       </c>
-      <c r="D40" t="n">
-        <v>80.55</v>
-      </c>
-      <c r="E40" t="n">
+      <c r="D16" t="n">
+        <v>79.37</v>
+      </c>
+      <c r="E16" t="n">
         <v>0</v>
       </c>
-      <c r="F40" t="n">
-        <v>80.55</v>
-      </c>
-      <c r="G40" t="inlineStr">
-        <is>
-          <t>2026-06-24 11:36:03</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" t="inlineStr">
-        <is>
-          <t>第 2 輪</t>
-        </is>
-      </c>
-      <c r="B41" t="inlineStr">
+      <c r="F16" t="n">
+        <v>79.37</v>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>2026-06-24 11:58:09</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>第 2 輪</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
         <is>
           <t>按鈕 8</t>
         </is>
       </c>
-      <c r="C41" t="inlineStr">
+      <c r="C17" t="inlineStr">
         <is>
           <t>CheckBox28_8</t>
         </is>
       </c>
-      <c r="D41" t="n">
-        <v>108.73</v>
-      </c>
-      <c r="E41" t="n">
+      <c r="D17" t="n">
+        <v>25.48</v>
+      </c>
+      <c r="E17" t="n">
         <v>0</v>
       </c>
-      <c r="F41" t="n">
-        <v>108.73</v>
-      </c>
-      <c r="G41" t="inlineStr">
-        <is>
-          <t>2026-06-24 11:36:05</t>
+      <c r="F17" t="n">
+        <v>25.48</v>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>2026-06-24 11:58:12</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: update report generate del: unused file fix: config and file name
</commit_message>
<xml_diff>
--- a/RF_All_Tests_Results_20260624.xlsx
+++ b/RF_All_Tests_Results_20260624.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G17"/>
+  <dimension ref="A1:G21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -468,21 +468,21 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>CheckBox28_1</t>
+          <t>CheckBoxSwNo</t>
         </is>
       </c>
       <c r="D2" t="n">
-        <v>0.2</v>
+        <v>0</v>
       </c>
       <c r="E2" t="n">
-        <v>160.93</v>
+        <v>0.04</v>
       </c>
       <c r="F2" t="n">
-        <v>160.93</v>
+        <v>0.04</v>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>2026-06-24 11:56:38</t>
+          <t>2026-06-24 15:43:26</t>
         </is>
       </c>
     </row>
@@ -499,21 +499,21 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>CheckBox28_2</t>
+          <t>CheckBoxSwNc</t>
         </is>
       </c>
       <c r="D3" t="n">
-        <v>111.99</v>
+        <v>55.49</v>
       </c>
       <c r="E3" t="n">
-        <v>111.99</v>
+        <v>110.45</v>
       </c>
       <c r="F3" t="n">
-        <v>111.99</v>
+        <v>110.45</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>2026-06-24 11:56:40</t>
+          <t>2026-06-24 15:43:28</t>
         </is>
       </c>
     </row>
@@ -530,21 +530,21 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>CheckBox28_3</t>
+          <t>CheckBox21</t>
         </is>
       </c>
       <c r="D4" t="n">
-        <v>53.51</v>
+        <v>0</v>
       </c>
       <c r="E4" t="n">
-        <v>102.4</v>
+        <v>166.53</v>
       </c>
       <c r="F4" t="n">
-        <v>102.4</v>
+        <v>166.53</v>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>2026-06-24 11:56:41</t>
+          <t>2026-06-24 15:43:29</t>
         </is>
       </c>
     </row>
@@ -561,21 +561,21 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>CheckBox28_4</t>
+          <t>CheckBox22</t>
         </is>
       </c>
       <c r="D5" t="n">
-        <v>109.74</v>
+        <v>0.11</v>
       </c>
       <c r="E5" t="n">
-        <v>109.74</v>
+        <v>55.17</v>
       </c>
       <c r="F5" t="n">
-        <v>109.74</v>
+        <v>55.17</v>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>2026-06-24 11:56:42</t>
+          <t>2026-06-24 15:43:30</t>
         </is>
       </c>
     </row>
@@ -592,21 +592,21 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>CheckBox28_5</t>
+          <t>CheckBox23</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>52.83</v>
+        <v>111.26</v>
       </c>
       <c r="E6" t="n">
-        <v>110.22</v>
+        <v>111.26</v>
       </c>
       <c r="F6" t="n">
-        <v>110.22</v>
+        <v>111.26</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>2026-06-24 11:56:43</t>
+          <t>2026-06-24 15:43:32</t>
         </is>
       </c>
     </row>
@@ -623,21 +623,21 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>CheckBox28_6</t>
+          <t>CheckBox24</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>111.83</v>
+        <v>108.48</v>
       </c>
       <c r="E7" t="n">
-        <v>111.83</v>
+        <v>108.48</v>
       </c>
       <c r="F7" t="n">
-        <v>111.83</v>
+        <v>108.48</v>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>2026-06-24 11:56:45</t>
+          <t>2026-06-24 15:43:33</t>
         </is>
       </c>
     </row>
@@ -654,21 +654,21 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>CheckBox28_7</t>
+          <t>CheckBox31</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>110.45</v>
+        <v>0</v>
       </c>
       <c r="E8" t="n">
-        <v>110.45</v>
+        <v>106.65</v>
       </c>
       <c r="F8" t="n">
-        <v>110.45</v>
+        <v>106.65</v>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>2026-06-24 11:56:46</t>
+          <t>2026-06-24 15:43:34</t>
         </is>
       </c>
     </row>
@@ -685,83 +685,83 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>CheckBox28_8</t>
+          <t>CheckBox32</t>
         </is>
       </c>
       <c r="D9" t="n">
-        <v>54.23</v>
+        <v>55.68</v>
       </c>
       <c r="E9" t="n">
-        <v>54.23</v>
+        <v>55.68</v>
       </c>
       <c r="F9" t="n">
-        <v>54.23</v>
+        <v>55.68</v>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>2026-06-24 11:56:47</t>
+          <t>2026-06-24 15:43:36</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>第 2 輪</t>
+          <t>第 1 輪</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>第 1 步</t>
+          <t>第 9 步</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>CheckBox28_1</t>
+          <t>CheckBox33</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>110.64</v>
+        <v>115.86</v>
       </c>
       <c r="E10" t="n">
-        <v>110.64</v>
+        <v>161.75</v>
       </c>
       <c r="F10" t="n">
-        <v>110.64</v>
+        <v>161.75</v>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>2026-06-24 11:56:49</t>
+          <t>2026-06-24 15:43:37</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>第 2 輪</t>
+          <t>第 1 輪</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>第 2 步</t>
+          <t>第 10 步</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>CheckBox28_2</t>
+          <t>CheckBox34</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>57.75</v>
+        <v>52.99</v>
       </c>
       <c r="E11" t="n">
-        <v>113.77</v>
+        <v>52.99</v>
       </c>
       <c r="F11" t="n">
-        <v>113.77</v>
+        <v>52.99</v>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>2026-06-24 11:56:50</t>
+          <t>2026-06-24 15:43:38</t>
         </is>
       </c>
     </row>
@@ -773,26 +773,26 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>第 3 步</t>
+          <t>第 1 步</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>CheckBox28_3</t>
+          <t>CheckBoxSwNo</t>
         </is>
       </c>
       <c r="D12" t="n">
-        <v>108.9</v>
+        <v>0</v>
       </c>
       <c r="E12" t="n">
-        <v>108.9</v>
+        <v>112.48</v>
       </c>
       <c r="F12" t="n">
-        <v>108.9</v>
+        <v>112.48</v>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>2026-06-24 11:56:51</t>
+          <t>2026-06-24 15:43:39</t>
         </is>
       </c>
     </row>
@@ -804,26 +804,26 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>第 4 步</t>
+          <t>第 2 步</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>CheckBox28_4</t>
+          <t>CheckBoxSwNc</t>
         </is>
       </c>
       <c r="D13" t="n">
-        <v>55.88</v>
+        <v>57.56</v>
       </c>
       <c r="E13" t="n">
-        <v>103.76</v>
+        <v>113.44</v>
       </c>
       <c r="F13" t="n">
-        <v>103.76</v>
+        <v>113.44</v>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>2026-06-24 11:56:53</t>
+          <t>2026-06-24 15:43:41</t>
         </is>
       </c>
     </row>
@@ -835,26 +835,26 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>第 5 步</t>
+          <t>第 3 步</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>CheckBox28_5</t>
+          <t>CheckBox21</t>
         </is>
       </c>
       <c r="D14" t="n">
-        <v>111.98</v>
+        <v>0</v>
       </c>
       <c r="E14" t="n">
-        <v>111.98</v>
+        <v>111.46</v>
       </c>
       <c r="F14" t="n">
-        <v>111.98</v>
+        <v>111.46</v>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>2026-06-24 11:56:54</t>
+          <t>2026-06-24 15:43:42</t>
         </is>
       </c>
     </row>
@@ -866,26 +866,26 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>第 6 步</t>
+          <t>第 4 步</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>CheckBox28_6</t>
+          <t>CheckBox22</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>111.02</v>
+        <v>107.66</v>
       </c>
       <c r="E15" t="n">
-        <v>111.02</v>
+        <v>107.66</v>
       </c>
       <c r="F15" t="n">
-        <v>111.02</v>
+        <v>107.66</v>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>2026-06-24 11:56:55</t>
+          <t>2026-06-24 15:43:43</t>
         </is>
       </c>
     </row>
@@ -897,26 +897,26 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>第 7 步</t>
+          <t>第 5 步</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>CheckBox28_7</t>
+          <t>CheckBox23</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>110.53</v>
+        <v>107.49</v>
       </c>
       <c r="E16" t="n">
-        <v>110.53</v>
+        <v>107.49</v>
       </c>
       <c r="F16" t="n">
-        <v>110.53</v>
+        <v>107.49</v>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>2026-06-24 11:56:56</t>
+          <t>2026-06-24 15:43:45</t>
         </is>
       </c>
     </row>
@@ -928,26 +928,150 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
+          <t>第 6 步</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>CheckBox24</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>56.09</v>
+      </c>
+      <c r="E17" t="n">
+        <v>103.58</v>
+      </c>
+      <c r="F17" t="n">
+        <v>103.58</v>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>2026-06-24 15:43:46</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>第 2 輪</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>第 7 步</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>CheckBox31</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
+        <v>0</v>
+      </c>
+      <c r="E18" t="n">
+        <v>110.09</v>
+      </c>
+      <c r="F18" t="n">
+        <v>110.09</v>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>2026-06-24 15:43:47</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>第 2 輪</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
           <t>第 8 步</t>
         </is>
       </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>CheckBox28_8</t>
-        </is>
-      </c>
-      <c r="D17" t="n">
-        <v>55.16</v>
-      </c>
-      <c r="E17" t="n">
-        <v>103.72</v>
-      </c>
-      <c r="F17" t="n">
-        <v>103.72</v>
-      </c>
-      <c r="G17" t="inlineStr">
-        <is>
-          <t>2026-06-24 11:56:58</t>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>CheckBox32</t>
+        </is>
+      </c>
+      <c r="D19" t="n">
+        <v>50.99</v>
+      </c>
+      <c r="E19" t="n">
+        <v>50.99</v>
+      </c>
+      <c r="F19" t="n">
+        <v>50.99</v>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>2026-06-24 15:43:49</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>第 2 輪</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>第 9 步</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>CheckBox33</t>
+        </is>
+      </c>
+      <c r="D20" t="n">
+        <v>110.93</v>
+      </c>
+      <c r="E20" t="n">
+        <v>110.93</v>
+      </c>
+      <c r="F20" t="n">
+        <v>110.93</v>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>2026-06-24 15:43:50</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>第 2 輪</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>第 10 步</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>CheckBox34</t>
+        </is>
+      </c>
+      <c r="D21" t="n">
+        <v>113.17</v>
+      </c>
+      <c r="E21" t="n">
+        <v>113.17</v>
+      </c>
+      <c r="F21" t="n">
+        <v>113.17</v>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>2026-06-24 15:43:51</t>
         </is>
       </c>
     </row>
@@ -962,7 +1086,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G25"/>
+  <dimension ref="A1:G31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1015,21 +1139,21 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>CheckBox28_1</t>
+          <t>CheckBoxSwNo</t>
         </is>
       </c>
       <c r="D2" t="n">
-        <v>0.06</v>
+        <v>0</v>
       </c>
       <c r="E2" t="n">
-        <v>212.51</v>
+        <v>0.42</v>
       </c>
       <c r="F2" t="n">
-        <v>212.51</v>
+        <v>0.42</v>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>2026-06-24 11:57:00</t>
+          <t>2026-06-24 15:43:54</t>
         </is>
       </c>
     </row>
@@ -1046,21 +1170,21 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>CheckBox28_2</t>
+          <t>CheckBoxSwNc</t>
         </is>
       </c>
       <c r="D3" t="n">
-        <v>110.66</v>
+        <v>0.06</v>
       </c>
       <c r="E3" t="n">
-        <v>110.66</v>
+        <v>54.4</v>
       </c>
       <c r="F3" t="n">
-        <v>110.66</v>
+        <v>54.4</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>2026-06-24 11:57:02</t>
+          <t>2026-06-24 15:43:55</t>
         </is>
       </c>
     </row>
@@ -1077,21 +1201,21 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>CheckBox28_1</t>
+          <t>CheckBoxSwNo</t>
         </is>
       </c>
       <c r="D4" t="n">
-        <v>109.29</v>
+        <v>53.24</v>
       </c>
       <c r="E4" t="n">
-        <v>109.29</v>
+        <v>108.77</v>
       </c>
       <c r="F4" t="n">
-        <v>109.29</v>
+        <v>108.77</v>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>2026-06-24 11:57:03</t>
+          <t>2026-06-24 15:43:56</t>
         </is>
       </c>
     </row>
@@ -1108,21 +1232,21 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>CheckBox28_3</t>
+          <t>CheckBox21</t>
         </is>
       </c>
       <c r="D5" t="n">
-        <v>53.95</v>
+        <v>0</v>
       </c>
       <c r="E5" t="n">
-        <v>102.41</v>
+        <v>111.49</v>
       </c>
       <c r="F5" t="n">
-        <v>102.41</v>
+        <v>111.49</v>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>2026-06-24 11:57:04</t>
+          <t>2026-06-24 15:43:58</t>
         </is>
       </c>
     </row>
@@ -1139,21 +1263,21 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>CheckBox28_4</t>
+          <t>CheckBox22</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>55.3</v>
+        <v>56.67</v>
       </c>
       <c r="E6" t="n">
-        <v>102.62</v>
+        <v>56.67</v>
       </c>
       <c r="F6" t="n">
-        <v>102.62</v>
+        <v>56.67</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>2026-06-24 11:57:06</t>
+          <t>2026-06-24 15:43:59</t>
         </is>
       </c>
     </row>
@@ -1170,21 +1294,21 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>CheckBox28_3</t>
+          <t>CheckBox21</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>57.84</v>
+        <v>110.28</v>
       </c>
       <c r="E7" t="n">
-        <v>114.5</v>
+        <v>110.28</v>
       </c>
       <c r="F7" t="n">
-        <v>114.5</v>
+        <v>110.28</v>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>2026-06-24 11:57:07</t>
+          <t>2026-06-24 15:44:00</t>
         </is>
       </c>
     </row>
@@ -1201,21 +1325,21 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>CheckBox28_5</t>
+          <t>CheckBox23</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>107.75</v>
+        <v>56.59</v>
       </c>
       <c r="E8" t="n">
-        <v>107.75</v>
+        <v>105.36</v>
       </c>
       <c r="F8" t="n">
-        <v>107.75</v>
+        <v>105.36</v>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>2026-06-24 11:57:08</t>
+          <t>2026-06-24 15:44:01</t>
         </is>
       </c>
     </row>
@@ -1232,21 +1356,21 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>CheckBox28_6</t>
+          <t>CheckBox24</t>
         </is>
       </c>
       <c r="D9" t="n">
-        <v>57.15</v>
+        <v>57.17</v>
       </c>
       <c r="E9" t="n">
-        <v>105.96</v>
+        <v>57.17</v>
       </c>
       <c r="F9" t="n">
-        <v>105.96</v>
+        <v>57.17</v>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>2026-06-24 11:57:09</t>
+          <t>2026-06-24 15:44:03</t>
         </is>
       </c>
     </row>
@@ -1263,21 +1387,21 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>CheckBox28_5</t>
+          <t>CheckBox23</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>109.35</v>
+        <v>50.95</v>
       </c>
       <c r="E10" t="n">
-        <v>109.35</v>
+        <v>99.67</v>
       </c>
       <c r="F10" t="n">
-        <v>109.35</v>
+        <v>99.67</v>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>2026-06-24 11:57:11</t>
+          <t>2026-06-24 15:44:04</t>
         </is>
       </c>
     </row>
@@ -1294,21 +1418,21 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>CheckBox28_7</t>
+          <t>CheckBox31</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>112.18</v>
+        <v>0</v>
       </c>
       <c r="E11" t="n">
-        <v>112.18</v>
+        <v>110.55</v>
       </c>
       <c r="F11" t="n">
-        <v>112.18</v>
+        <v>110.55</v>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>2026-06-24 11:57:12</t>
+          <t>2026-06-24 15:44:05</t>
         </is>
       </c>
     </row>
@@ -1325,21 +1449,21 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>CheckBox28_8</t>
+          <t>CheckBox32</t>
         </is>
       </c>
       <c r="D12" t="n">
-        <v>108.52</v>
+        <v>0.17</v>
       </c>
       <c r="E12" t="n">
-        <v>108.52</v>
+        <v>50.98</v>
       </c>
       <c r="F12" t="n">
-        <v>108.52</v>
+        <v>50.98</v>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>2026-06-24 11:57:13</t>
+          <t>2026-06-24 15:44:07</t>
         </is>
       </c>
     </row>
@@ -1356,114 +1480,114 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>CheckBox28_7</t>
+          <t>CheckBox31</t>
         </is>
       </c>
       <c r="D13" t="n">
-        <v>54.66</v>
+        <v>110.46</v>
       </c>
       <c r="E13" t="n">
-        <v>103.32</v>
+        <v>110.46</v>
       </c>
       <c r="F13" t="n">
-        <v>103.32</v>
+        <v>110.46</v>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>2026-06-24 11:57:15</t>
+          <t>2026-06-24 15:44:08</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>第 2 輪</t>
+          <t>第 1 輪</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>第 1 步 (鈕 1)</t>
+          <t>第 13 步 (鈕 9)</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>CheckBox28_1</t>
+          <t>CheckBox33</t>
         </is>
       </c>
       <c r="D14" t="n">
-        <v>58.82</v>
+        <v>0.1</v>
       </c>
       <c r="E14" t="n">
-        <v>106.77</v>
+        <v>50.71</v>
       </c>
       <c r="F14" t="n">
-        <v>106.77</v>
+        <v>50.71</v>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>2026-06-24 11:57:16</t>
+          <t>2026-06-24 15:44:09</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>第 2 輪</t>
+          <t>第 1 輪</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>第 2 步 (鈕 2)</t>
+          <t>第 14 步 (鈕 10)</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>CheckBox28_2</t>
+          <t>CheckBox34</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>52.84</v>
+        <v>52.09</v>
       </c>
       <c r="E15" t="n">
-        <v>102.35</v>
+        <v>100.77</v>
       </c>
       <c r="F15" t="n">
-        <v>102.35</v>
+        <v>100.77</v>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>2026-06-24 11:57:17</t>
+          <t>2026-06-24 15:44:10</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>第 2 輪</t>
+          <t>第 1 輪</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>第 3 步 (鈕 1)</t>
+          <t>第 15 步 (鈕 9)</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>CheckBox28_1</t>
+          <t>CheckBox33</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>54.68</v>
+        <v>55.45</v>
       </c>
       <c r="E16" t="n">
-        <v>103.02</v>
+        <v>101.74</v>
       </c>
       <c r="F16" t="n">
-        <v>103.02</v>
+        <v>101.74</v>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>2026-06-24 11:57:19</t>
+          <t>2026-06-24 15:44:12</t>
         </is>
       </c>
     </row>
@@ -1475,26 +1599,26 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>第 4 步 (鈕 3)</t>
+          <t>第 1 步 (鈕 1)</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>CheckBox28_3</t>
+          <t>CheckBoxSwNo</t>
         </is>
       </c>
       <c r="D17" t="n">
-        <v>54.93</v>
+        <v>0</v>
       </c>
       <c r="E17" t="n">
-        <v>111.7</v>
+        <v>0</v>
       </c>
       <c r="F17" t="n">
-        <v>111.7</v>
+        <v>0</v>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>2026-06-24 11:57:20</t>
+          <t>2026-06-24 15:44:15</t>
         </is>
       </c>
     </row>
@@ -1506,26 +1630,26 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>第 5 步 (鈕 4)</t>
+          <t>第 2 步 (鈕 2)</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>CheckBox28_4</t>
+          <t>CheckBoxSwNc</t>
         </is>
       </c>
       <c r="D18" t="n">
-        <v>52.53</v>
+        <v>0.1</v>
       </c>
       <c r="E18" t="n">
-        <v>101.09</v>
+        <v>0</v>
       </c>
       <c r="F18" t="n">
-        <v>101.09</v>
+        <v>0</v>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>2026-06-24 11:57:21</t>
+          <t>2026-06-24 15:44:18</t>
         </is>
       </c>
     </row>
@@ -1537,26 +1661,26 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>第 6 步 (鈕 3)</t>
+          <t>第 3 步 (鈕 1)</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>CheckBox28_3</t>
+          <t>CheckBoxSwNo</t>
         </is>
       </c>
       <c r="D19" t="n">
-        <v>53.68</v>
+        <v>0</v>
       </c>
       <c r="E19" t="n">
-        <v>108.66</v>
+        <v>0</v>
       </c>
       <c r="F19" t="n">
-        <v>108.66</v>
+        <v>0</v>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>2026-06-24 11:57:22</t>
+          <t>2026-06-24 15:44:21</t>
         </is>
       </c>
     </row>
@@ -1568,26 +1692,26 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>第 7 步 (鈕 5)</t>
+          <t>第 4 步 (鈕 3)</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>CheckBox28_5</t>
+          <t>CheckBox21</t>
         </is>
       </c>
       <c r="D20" t="n">
-        <v>112.53</v>
+        <v>0.06</v>
       </c>
       <c r="E20" t="n">
-        <v>112.53</v>
+        <v>198.68</v>
       </c>
       <c r="F20" t="n">
-        <v>112.53</v>
+        <v>198.68</v>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>2026-06-24 11:57:24</t>
+          <t>2026-06-24 15:44:23</t>
         </is>
       </c>
     </row>
@@ -1599,26 +1723,26 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>第 8 步 (鈕 6)</t>
+          <t>第 5 步 (鈕 4)</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>CheckBox28_6</t>
+          <t>CheckBox22</t>
         </is>
       </c>
       <c r="D21" t="n">
-        <v>59.28</v>
+        <v>57.94</v>
       </c>
       <c r="E21" t="n">
-        <v>107.5</v>
+        <v>105.2</v>
       </c>
       <c r="F21" t="n">
-        <v>107.5</v>
+        <v>105.2</v>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>2026-06-24 11:57:25</t>
+          <t>2026-06-24 15:44:24</t>
         </is>
       </c>
     </row>
@@ -1630,26 +1754,26 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>第 9 步 (鈕 5)</t>
+          <t>第 6 步 (鈕 3)</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>CheckBox28_5</t>
+          <t>CheckBox21</t>
         </is>
       </c>
       <c r="D22" t="n">
-        <v>108.04</v>
+        <v>58.72</v>
       </c>
       <c r="E22" t="n">
-        <v>108.04</v>
+        <v>58.72</v>
       </c>
       <c r="F22" t="n">
-        <v>108.04</v>
+        <v>58.72</v>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>2026-06-24 11:57:26</t>
+          <t>2026-06-24 15:44:26</t>
         </is>
       </c>
     </row>
@@ -1661,26 +1785,26 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>第 10 步 (鈕 7)</t>
+          <t>第 7 步 (鈕 5)</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>CheckBox28_7</t>
+          <t>CheckBox23</t>
         </is>
       </c>
       <c r="D23" t="n">
-        <v>55.58</v>
+        <v>59.28</v>
       </c>
       <c r="E23" t="n">
-        <v>104.06</v>
+        <v>59.28</v>
       </c>
       <c r="F23" t="n">
-        <v>104.06</v>
+        <v>59.28</v>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>2026-06-24 11:57:28</t>
+          <t>2026-06-24 15:44:27</t>
         </is>
       </c>
     </row>
@@ -1692,26 +1816,26 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>第 11 步 (鈕 8)</t>
+          <t>第 8 步 (鈕 6)</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>CheckBox28_8</t>
+          <t>CheckBox24</t>
         </is>
       </c>
       <c r="D24" t="n">
-        <v>53.92</v>
+        <v>54.1</v>
       </c>
       <c r="E24" t="n">
-        <v>103.28</v>
+        <v>103.24</v>
       </c>
       <c r="F24" t="n">
-        <v>103.28</v>
+        <v>103.24</v>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>2026-06-24 11:57:29</t>
+          <t>2026-06-24 15:44:28</t>
         </is>
       </c>
     </row>
@@ -1723,26 +1847,212 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
+          <t>第 9 步 (鈕 5)</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>CheckBox23</t>
+        </is>
+      </c>
+      <c r="D25" t="n">
+        <v>53.4</v>
+      </c>
+      <c r="E25" t="n">
+        <v>53.4</v>
+      </c>
+      <c r="F25" t="n">
+        <v>53.4</v>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>2026-06-24 15:44:29</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>第 2 輪</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>第 10 步 (鈕 7)</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>CheckBox31</t>
+        </is>
+      </c>
+      <c r="D26" t="n">
+        <v>0</v>
+      </c>
+      <c r="E26" t="n">
+        <v>110.92</v>
+      </c>
+      <c r="F26" t="n">
+        <v>110.92</v>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>2026-06-24 15:44:31</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>第 2 輪</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>第 11 步 (鈕 8)</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>CheckBox32</t>
+        </is>
+      </c>
+      <c r="D27" t="n">
+        <v>56.62</v>
+      </c>
+      <c r="E27" t="n">
+        <v>104.25</v>
+      </c>
+      <c r="F27" t="n">
+        <v>104.25</v>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>2026-06-24 15:44:32</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>第 2 輪</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
           <t>第 12 步 (鈕 7)</t>
         </is>
       </c>
-      <c r="C25" t="inlineStr">
-        <is>
-          <t>CheckBox28_7</t>
-        </is>
-      </c>
-      <c r="D25" t="n">
-        <v>55.41</v>
-      </c>
-      <c r="E25" t="n">
-        <v>104.06</v>
-      </c>
-      <c r="F25" t="n">
-        <v>104.06</v>
-      </c>
-      <c r="G25" t="inlineStr">
-        <is>
-          <t>2026-06-24 11:57:30</t>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>CheckBox31</t>
+        </is>
+      </c>
+      <c r="D28" t="n">
+        <v>55.37</v>
+      </c>
+      <c r="E28" t="n">
+        <v>55.37</v>
+      </c>
+      <c r="F28" t="n">
+        <v>55.37</v>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>2026-06-24 15:44:33</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>第 2 輪</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>第 13 步 (鈕 9)</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>CheckBox33</t>
+        </is>
+      </c>
+      <c r="D29" t="n">
+        <v>56.65</v>
+      </c>
+      <c r="E29" t="n">
+        <v>103.03</v>
+      </c>
+      <c r="F29" t="n">
+        <v>103.03</v>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>2026-06-24 15:44:35</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>第 2 輪</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>第 14 步 (鈕 10)</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>CheckBox34</t>
+        </is>
+      </c>
+      <c r="D30" t="n">
+        <v>108.18</v>
+      </c>
+      <c r="E30" t="n">
+        <v>108.18</v>
+      </c>
+      <c r="F30" t="n">
+        <v>108.18</v>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>2026-06-24 15:44:36</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>第 2 輪</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>第 15 步 (鈕 9)</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>CheckBox33</t>
+        </is>
+      </c>
+      <c r="D31" t="n">
+        <v>56.66</v>
+      </c>
+      <c r="E31" t="n">
+        <v>56.66</v>
+      </c>
+      <c r="F31" t="n">
+        <v>56.66</v>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>2026-06-24 15:44:37</t>
         </is>
       </c>
     </row>
@@ -1757,7 +2067,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G17"/>
+  <dimension ref="A1:G21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1810,7 +2120,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>CheckBox28_1</t>
+          <t>CheckBoxSwNo</t>
         </is>
       </c>
       <c r="D2" t="n">
@@ -1824,7 +2134,7 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>2026-06-24 11:57:33</t>
+          <t>2026-06-24 15:44:40</t>
         </is>
       </c>
     </row>
@@ -1841,21 +2151,21 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>CheckBox28_2</t>
+          <t>CheckBoxSwNc</t>
         </is>
       </c>
       <c r="D3" t="n">
-        <v>57.17</v>
+        <v>0</v>
       </c>
       <c r="E3" t="n">
         <v>0</v>
       </c>
       <c r="F3" t="n">
-        <v>57.18</v>
+        <v>0</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>2026-06-24 11:57:35</t>
+          <t>2026-06-24 15:44:47</t>
         </is>
       </c>
     </row>
@@ -1872,21 +2182,21 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>CheckBox28_3</t>
+          <t>CheckBox21</t>
         </is>
       </c>
       <c r="D4" t="n">
-        <v>52.71</v>
+        <v>135.26</v>
       </c>
       <c r="E4" t="n">
         <v>0</v>
       </c>
       <c r="F4" t="n">
-        <v>52.72</v>
+        <v>135.26</v>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>2026-06-24 11:57:38</t>
+          <t>2026-06-24 15:44:49</t>
         </is>
       </c>
     </row>
@@ -1903,21 +2213,21 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>CheckBox28_4</t>
+          <t>CheckBox22</t>
         </is>
       </c>
       <c r="D5" t="n">
-        <v>24.21</v>
+        <v>81.54000000000001</v>
       </c>
       <c r="E5" t="n">
         <v>0</v>
       </c>
       <c r="F5" t="n">
-        <v>24.21</v>
+        <v>81.54000000000001</v>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>2026-06-24 11:57:41</t>
+          <t>2026-06-24 15:44:52</t>
         </is>
       </c>
     </row>
@@ -1934,21 +2244,21 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>CheckBox28_5</t>
+          <t>CheckBox23</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>30.08</v>
+        <v>24.97</v>
       </c>
       <c r="E6" t="n">
         <v>0</v>
       </c>
       <c r="F6" t="n">
-        <v>30.08</v>
+        <v>24.97</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>2026-06-24 11:57:43</t>
+          <t>2026-06-24 15:44:55</t>
         </is>
       </c>
     </row>
@@ -1965,21 +2275,21 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>CheckBox28_6</t>
+          <t>CheckBox24</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>26.22</v>
+        <v>26.12</v>
       </c>
       <c r="E7" t="n">
         <v>0</v>
       </c>
       <c r="F7" t="n">
-        <v>26.23</v>
+        <v>26.12</v>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>2026-06-24 11:57:46</t>
+          <t>2026-06-24 15:44:57</t>
         </is>
       </c>
     </row>
@@ -1996,21 +2306,21 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>CheckBox28_7</t>
+          <t>CheckBox31</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>56.01</v>
+        <v>24.52</v>
       </c>
       <c r="E8" t="n">
         <v>0</v>
       </c>
       <c r="F8" t="n">
-        <v>56.01</v>
+        <v>24.52</v>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>2026-06-24 11:57:48</t>
+          <t>2026-06-24 15:45:00</t>
         </is>
       </c>
     </row>
@@ -2027,83 +2337,83 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>CheckBox28_8</t>
+          <t>CheckBox32</t>
         </is>
       </c>
       <c r="D9" t="n">
-        <v>55.16</v>
+        <v>30.02</v>
       </c>
       <c r="E9" t="n">
         <v>0</v>
       </c>
       <c r="F9" t="n">
-        <v>55.16</v>
+        <v>30.02</v>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>2026-06-24 11:57:51</t>
+          <t>2026-06-24 15:45:02</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>第 2 輪</t>
+          <t>第 1 輪</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>按鈕 1</t>
+          <t>按鈕 9</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>CheckBox28_1</t>
+          <t>CheckBox33</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>81.65000000000001</v>
+        <v>27.26</v>
       </c>
       <c r="E10" t="n">
         <v>0</v>
       </c>
       <c r="F10" t="n">
-        <v>81.65000000000001</v>
+        <v>27.27</v>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>2026-06-24 11:57:54</t>
+          <t>2026-06-24 15:45:05</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>第 2 輪</t>
+          <t>第 1 輪</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>按鈕 2</t>
+          <t>按鈕 10</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>CheckBox28_2</t>
+          <t>CheckBox34</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>23.64</v>
+        <v>26.21</v>
       </c>
       <c r="E11" t="n">
         <v>0</v>
       </c>
       <c r="F11" t="n">
-        <v>23.65</v>
+        <v>26.21</v>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>2026-06-24 11:57:56</t>
+          <t>2026-06-24 15:45:08</t>
         </is>
       </c>
     </row>
@@ -2115,26 +2425,26 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>按鈕 3</t>
+          <t>按鈕 1</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>CheckBox28_3</t>
+          <t>CheckBoxSwNo</t>
         </is>
       </c>
       <c r="D12" t="n">
-        <v>58.75</v>
+        <v>0</v>
       </c>
       <c r="E12" t="n">
         <v>0</v>
       </c>
       <c r="F12" t="n">
-        <v>58.75</v>
+        <v>0</v>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>2026-06-24 11:57:59</t>
+          <t>2026-06-24 15:45:10</t>
         </is>
       </c>
     </row>
@@ -2146,26 +2456,26 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>按鈕 4</t>
+          <t>按鈕 2</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>CheckBox28_4</t>
+          <t>CheckBoxSwNc</t>
         </is>
       </c>
       <c r="D13" t="n">
-        <v>56.82</v>
+        <v>0</v>
       </c>
       <c r="E13" t="n">
-        <v>111.74</v>
+        <v>0</v>
       </c>
       <c r="F13" t="n">
-        <v>168.56</v>
+        <v>0</v>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>2026-06-24 11:58:02</t>
+          <t>2026-06-24 15:45:15</t>
         </is>
       </c>
     </row>
@@ -2177,26 +2487,26 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>按鈕 5</t>
+          <t>按鈕 3</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>CheckBox28_5</t>
+          <t>CheckBox21</t>
         </is>
       </c>
       <c r="D14" t="n">
-        <v>137.75</v>
+        <v>0</v>
       </c>
       <c r="E14" t="n">
         <v>0</v>
       </c>
       <c r="F14" t="n">
-        <v>137.75</v>
+        <v>0</v>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>2026-06-24 11:58:04</t>
+          <t>2026-06-24 15:45:18</t>
         </is>
       </c>
     </row>
@@ -2208,26 +2518,26 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>按鈕 6</t>
+          <t>按鈕 4</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>CheckBox28_6</t>
+          <t>CheckBox22</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>0</v>
+        <v>56.05</v>
       </c>
       <c r="E15" t="n">
         <v>0</v>
       </c>
       <c r="F15" t="n">
-        <v>0</v>
+        <v>56.05</v>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>2026-06-24 11:58:07</t>
+          <t>2026-06-24 15:45:20</t>
         </is>
       </c>
     </row>
@@ -2239,26 +2549,26 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>按鈕 7</t>
+          <t>按鈕 5</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>CheckBox28_7</t>
+          <t>CheckBox23</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>79.37</v>
+        <v>27.44</v>
       </c>
       <c r="E16" t="n">
         <v>0</v>
       </c>
       <c r="F16" t="n">
-        <v>79.37</v>
+        <v>27.44</v>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>2026-06-24 11:58:09</t>
+          <t>2026-06-24 15:45:23</t>
         </is>
       </c>
     </row>
@@ -2270,26 +2580,150 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
+          <t>按鈕 6</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>CheckBox24</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>54.17</v>
+      </c>
+      <c r="E17" t="n">
+        <v>0</v>
+      </c>
+      <c r="F17" t="n">
+        <v>54.17</v>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>2026-06-24 15:45:26</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>第 2 輪</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>按鈕 7</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>CheckBox31</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
+        <v>26.01</v>
+      </c>
+      <c r="E18" t="n">
+        <v>0</v>
+      </c>
+      <c r="F18" t="n">
+        <v>26.01</v>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>2026-06-24 15:45:28</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>第 2 輪</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
           <t>按鈕 8</t>
         </is>
       </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>CheckBox28_8</t>
-        </is>
-      </c>
-      <c r="D17" t="n">
-        <v>25.48</v>
-      </c>
-      <c r="E17" t="n">
-        <v>0</v>
-      </c>
-      <c r="F17" t="n">
-        <v>25.48</v>
-      </c>
-      <c r="G17" t="inlineStr">
-        <is>
-          <t>2026-06-24 11:58:12</t>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>CheckBox32</t>
+        </is>
+      </c>
+      <c r="D19" t="n">
+        <v>83.23999999999999</v>
+      </c>
+      <c r="E19" t="n">
+        <v>0</v>
+      </c>
+      <c r="F19" t="n">
+        <v>83.23999999999999</v>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>2026-06-24 15:45:31</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>第 2 輪</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>按鈕 9</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>CheckBox33</t>
+        </is>
+      </c>
+      <c r="D20" t="n">
+        <v>27.75</v>
+      </c>
+      <c r="E20" t="n">
+        <v>0</v>
+      </c>
+      <c r="F20" t="n">
+        <v>27.75</v>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>2026-06-24 15:45:33</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>第 2 輪</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>按鈕 10</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>CheckBox34</t>
+        </is>
+      </c>
+      <c r="D21" t="n">
+        <v>28.68</v>
+      </c>
+      <c r="E21" t="n">
+        <v>0</v>
+      </c>
+      <c r="F21" t="n">
+        <v>28.68</v>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>2026-06-24 15:45:36</t>
         </is>
       </c>
     </row>

</xml_diff>